<commit_message>
implemented axis from 0
</commit_message>
<xml_diff>
--- a/data/APT_Tungsten_China.xlsx
+++ b/data/APT_Tungsten_China.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr checkCompatibility="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{481345B0-5298-4922-A209-4478623E1AC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{AE462AAD-0355-4FE4-B259-6F1180EB71EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="780" yWindow="780" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="2" r:id="rId1"/>
@@ -841,7 +841,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:BLL4"/>
+  <dimension ref="A1:BLS4"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col min="186" max="186" width="10.375" customWidth="1"/>
@@ -1006,9 +1006,10 @@
     <col min="1524" max="1524" width="9.5" customWidth="1"/>
     <col min="1542" max="1542" width="9.875" customWidth="1"/>
     <col min="1570" max="1570" width="10" customWidth="1"/>
+    <col min="1680" max="1683" width="9" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1676">
+    <row r="1" spans="1:1683">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -6037,8 +6038,29 @@
       <c r="BLL1" s="4">
         <v>46289</v>
       </c>
+      <c r="BLM1" s="4">
+        <v>46293</v>
+      </c>
+      <c r="BLN1" s="4">
+        <v>46294</v>
+      </c>
+      <c r="BLO1" s="4">
+        <v>46295</v>
+      </c>
+      <c r="BLP1" s="4">
+        <v>46303</v>
+      </c>
+      <c r="BLQ1" s="4">
+        <v>46304</v>
+      </c>
+      <c r="BLR1" s="4">
+        <v>46305</v>
+      </c>
+      <c r="BLS1" s="4">
+        <v>46307</v>
+      </c>
     </row>
-    <row r="2" spans="1:1676" ht="14.25">
+    <row r="2" spans="1:1683" ht="14.25">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
@@ -11067,8 +11089,29 @@
       <c r="BLL2" s="6">
         <v>570</v>
       </c>
+      <c r="BLM2" s="6">
+        <v>570</v>
+      </c>
+      <c r="BLN2" s="6">
+        <v>560</v>
+      </c>
+      <c r="BLO2" s="6">
+        <v>550</v>
+      </c>
+      <c r="BLP2" s="6">
+        <v>540</v>
+      </c>
+      <c r="BLQ2" s="6">
+        <v>540</v>
+      </c>
+      <c r="BLR2" s="6">
+        <v>525</v>
+      </c>
+      <c r="BLS2" s="6">
+        <v>510</v>
+      </c>
     </row>
-    <row r="3" spans="1:1676" s="3" customFormat="1" ht="14.25">
+    <row r="3" spans="1:1683" s="3" customFormat="1" ht="14.25">
       <c r="A3" s="2" t="s">
         <v>2</v>
       </c>
@@ -16794,738 +16837,766 @@
       </c>
       <c r="BEL3" s="14">
         <f>AVERAGE(BEL2:CAE2)</f>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BEM3" s="9">
         <f t="shared" ref="BEM3:BER3" si="570">BEL3</f>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BEN3" s="9">
         <f t="shared" si="570"/>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BEO3" s="9">
         <f t="shared" si="570"/>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BEP3" s="9">
         <f t="shared" si="570"/>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BEQ3" s="9">
         <f t="shared" si="570"/>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BER3" s="9">
         <f t="shared" si="570"/>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BES3" s="9">
         <f t="shared" ref="BES3" si="571">BER3</f>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BET3" s="9">
         <f t="shared" ref="BET3" si="572">BES3</f>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BEU3" s="9">
         <f t="shared" ref="BEU3:BEW3" si="573">BET3</f>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BEV3" s="9">
         <f t="shared" si="573"/>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BEW3" s="9">
         <f t="shared" si="573"/>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BEX3" s="9">
         <f t="shared" ref="BEX3" si="574">BEW3</f>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BEY3" s="9">
         <f t="shared" ref="BEY3:BEZ3" si="575">BEX3</f>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BEZ3" s="9">
         <f t="shared" si="575"/>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BFA3" s="9">
         <f t="shared" ref="BFA3" si="576">BEZ3</f>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BFB3" s="9">
         <f t="shared" ref="BFB3" si="577">BFA3</f>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BFC3" s="9">
         <f t="shared" ref="BFC3" si="578">BFB3</f>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BFD3" s="9">
         <f t="shared" ref="BFD3:BFF3" si="579">BFC3</f>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BFE3" s="9">
         <f t="shared" si="579"/>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BFF3" s="9">
         <f t="shared" si="579"/>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BFG3" s="9">
         <f t="shared" ref="BFG3" si="580">BFF3</f>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BFH3" s="9">
         <f t="shared" ref="BFH3" si="581">BFG3</f>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BFI3" s="9">
         <f t="shared" ref="BFI3" si="582">BFH3</f>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BFJ3" s="9">
         <f t="shared" ref="BFJ3:BFL3" si="583">BFI3</f>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BFK3" s="9">
         <f t="shared" si="583"/>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BFL3" s="9">
         <f t="shared" si="583"/>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BFM3" s="9">
         <f t="shared" ref="BFM3" si="584">BFL3</f>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BFN3" s="9">
         <f t="shared" ref="BFN3" si="585">BFM3</f>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BFO3" s="9">
         <f t="shared" ref="BFO3" si="586">BFN3</f>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BFP3" s="9">
         <f t="shared" ref="BFP3" si="587">BFO3</f>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BFQ3" s="9">
         <f t="shared" ref="BFQ3" si="588">BFP3</f>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BFR3" s="9">
         <f t="shared" ref="BFR3:BGD3" si="589">BFQ3</f>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BFS3" s="9">
         <f t="shared" si="589"/>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BFT3" s="9">
         <f t="shared" si="589"/>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BFU3" s="9">
         <f t="shared" si="589"/>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BFV3" s="9">
         <f t="shared" si="589"/>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BFW3" s="9">
         <f t="shared" si="589"/>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BFX3" s="9">
         <f t="shared" si="589"/>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BFY3" s="9">
         <f t="shared" si="589"/>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BFZ3" s="9">
         <f t="shared" si="589"/>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BGA3" s="9">
         <f t="shared" si="589"/>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BGB3" s="9">
         <f t="shared" si="589"/>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BGC3" s="9">
         <f t="shared" si="589"/>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BGD3" s="9">
         <f t="shared" si="589"/>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BGE3" s="9">
         <f t="shared" ref="BGE3" si="590">BGD3</f>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BGF3" s="9">
         <f t="shared" ref="BGF3:BGN3" si="591">BGE3</f>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BGG3" s="9">
         <f t="shared" si="591"/>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BGH3" s="9">
         <f t="shared" si="591"/>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BGI3" s="9">
         <f t="shared" si="591"/>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BGJ3" s="9">
         <f t="shared" si="591"/>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BGK3" s="9">
         <f t="shared" si="591"/>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BGL3" s="9">
         <f t="shared" si="591"/>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BGM3" s="9">
         <f t="shared" si="591"/>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BGN3" s="9">
         <f t="shared" si="591"/>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BGO3" s="9">
         <f t="shared" ref="BGO3" si="592">BGN3</f>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BGP3" s="9">
         <f t="shared" ref="BGP3:BGS3" si="593">BGO3</f>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BGQ3" s="9">
         <f t="shared" si="593"/>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BGR3" s="9">
         <f t="shared" si="593"/>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BGS3" s="9">
         <f t="shared" si="593"/>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BGT3" s="9">
         <f t="shared" ref="BGT3" si="594">BGS3</f>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BGU3" s="9">
         <f t="shared" ref="BGU3:BGY3" si="595">BGT3</f>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BGV3" s="9">
         <f t="shared" si="595"/>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BGW3" s="9">
         <f t="shared" si="595"/>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BGX3" s="9">
         <f t="shared" si="595"/>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BGY3" s="9">
         <f t="shared" si="595"/>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BGZ3" s="9">
         <f t="shared" ref="BGZ3" si="596">BGY3</f>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BHA3" s="9">
         <f t="shared" ref="BHA3" si="597">BGZ3</f>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BHB3" s="9">
         <f t="shared" ref="BHB3" si="598">BHA3</f>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BHC3" s="9">
         <f t="shared" ref="BHC3:BHE3" si="599">BHB3</f>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BHD3" s="9">
         <f t="shared" si="599"/>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BHE3" s="9">
         <f t="shared" si="599"/>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BHF3" s="9">
         <f t="shared" ref="BHF3" si="600">BHE3</f>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BHG3" s="9">
         <f t="shared" ref="BHG3" si="601">BHF3</f>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BHH3" s="9">
         <f t="shared" ref="BHH3" si="602">BHG3</f>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BHI3" s="9">
         <f t="shared" ref="BHI3:BHJ3" si="603">BHH3</f>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BHJ3" s="9">
         <f t="shared" si="603"/>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BHK3" s="9">
         <f t="shared" ref="BHK3" si="604">BHJ3</f>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BHL3" s="9">
         <f t="shared" ref="BHL3:BHR3" si="605">BHK3</f>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BHM3" s="9">
         <f t="shared" si="605"/>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BHN3" s="9">
         <f t="shared" si="605"/>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BHO3" s="9">
         <f t="shared" si="605"/>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BHP3" s="9">
         <f t="shared" si="605"/>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BHQ3" s="9">
         <f t="shared" si="605"/>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BHR3" s="9">
         <f t="shared" si="605"/>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BHS3" s="9">
         <f t="shared" ref="BHS3" si="606">BHR3</f>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BHT3" s="9">
         <f t="shared" ref="BHT3" si="607">BHS3</f>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BHU3" s="9">
         <f t="shared" ref="BHU3" si="608">BHT3</f>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BHV3" s="9">
         <f t="shared" ref="BHV3:BHW3" si="609">BHU3</f>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BHW3" s="9">
         <f t="shared" si="609"/>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BHX3" s="9">
         <f t="shared" ref="BHX3" si="610">BHW3</f>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BHY3" s="9">
         <f t="shared" ref="BHY3" si="611">BHX3</f>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BHZ3" s="9">
         <f t="shared" ref="BHZ3:BIJ3" si="612">BHY3</f>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BIA3" s="9">
         <f t="shared" si="612"/>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BIB3" s="9">
         <f t="shared" si="612"/>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BIC3" s="9">
         <f t="shared" si="612"/>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BID3" s="9">
         <f t="shared" si="612"/>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BIE3" s="9">
         <f t="shared" si="612"/>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BIF3" s="9">
         <f t="shared" si="612"/>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BIG3" s="9">
         <f t="shared" si="612"/>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BIH3" s="9">
         <f t="shared" si="612"/>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BII3" s="9">
         <f t="shared" si="612"/>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BIJ3" s="9">
         <f t="shared" si="612"/>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BIK3" s="9">
         <f t="shared" ref="BIK3" si="613">BIJ3</f>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BIL3" s="9">
         <f t="shared" ref="BIL3" si="614">BIK3</f>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BIM3" s="9">
         <f t="shared" ref="BIM3" si="615">BIL3</f>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BIN3" s="9">
         <f t="shared" ref="BIN3:BIO3" si="616">BIM3</f>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BIO3" s="9">
         <f t="shared" si="616"/>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BIP3" s="9">
         <f t="shared" ref="BIP3" si="617">BIO3</f>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BIQ3" s="9">
         <f t="shared" ref="BIQ3:BJF3" si="618">BIP3</f>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BIR3" s="9">
         <f t="shared" si="618"/>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BIS3" s="9">
         <f t="shared" si="618"/>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BIT3" s="9">
         <f t="shared" si="618"/>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BIU3" s="9">
         <f t="shared" si="618"/>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BIV3" s="9">
         <f t="shared" si="618"/>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BIW3" s="9">
         <f t="shared" si="618"/>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BIX3" s="9">
         <f t="shared" si="618"/>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BIY3" s="9">
         <f t="shared" si="618"/>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BIZ3" s="9">
         <f t="shared" si="618"/>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BJA3" s="9">
         <f t="shared" si="618"/>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BJB3" s="9">
         <f t="shared" si="618"/>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BJC3" s="9">
         <f t="shared" si="618"/>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BJD3" s="9">
         <f t="shared" si="618"/>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BJE3" s="9">
         <f t="shared" si="618"/>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BJF3" s="9">
         <f t="shared" si="618"/>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BJG3" s="9">
         <f t="shared" ref="BJG3" si="619">BJF3</f>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BJH3" s="9">
         <f t="shared" ref="BJH3" si="620">BJG3</f>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BJI3" s="9">
         <f t="shared" ref="BJI3" si="621">BJH3</f>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BJJ3" s="9">
         <f t="shared" ref="BJJ3" si="622">BJI3</f>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BJK3" s="9">
         <f t="shared" ref="BJK3:BJM3" si="623">BJJ3</f>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BJL3" s="9">
         <f t="shared" si="623"/>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BJM3" s="9">
         <f t="shared" si="623"/>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BJN3" s="9">
         <f t="shared" ref="BJN3" si="624">BJM3</f>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BJO3" s="9">
         <f t="shared" ref="BJO3:BJR3" si="625">BJN3</f>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BJP3" s="9">
         <f t="shared" si="625"/>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BJQ3" s="9">
         <f t="shared" si="625"/>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BJR3" s="9">
         <f t="shared" si="625"/>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BJS3" s="9">
         <f t="shared" ref="BJS3" si="626">BJR3</f>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BJT3" s="9">
         <f t="shared" ref="BJT3:BKE3" si="627">BJS3</f>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BJU3" s="9">
         <f t="shared" si="627"/>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BJV3" s="9">
         <f t="shared" si="627"/>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BJW3" s="9">
         <f t="shared" si="627"/>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BJX3" s="9">
         <f t="shared" si="627"/>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BJY3" s="9">
         <f t="shared" si="627"/>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BJZ3" s="9">
         <f t="shared" si="627"/>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BKA3" s="9">
         <f t="shared" si="627"/>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BKB3" s="9">
         <f t="shared" si="627"/>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BKC3" s="9">
         <f t="shared" si="627"/>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BKD3" s="9">
         <f t="shared" si="627"/>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BKE3" s="9">
         <f t="shared" si="627"/>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BKF3" s="9">
         <f t="shared" ref="BKF3" si="628">BKE3</f>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BKG3" s="9">
         <f t="shared" ref="BKG3" si="629">BKF3</f>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BKH3" s="9">
         <f t="shared" ref="BKH3" si="630">BKG3</f>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BKI3" s="9">
         <f t="shared" ref="BKI3" si="631">BKH3</f>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BKJ3" s="9">
         <f t="shared" ref="BKJ3" si="632">BKI3</f>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BKK3" s="9">
         <f t="shared" ref="BKK3" si="633">BKJ3</f>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BKL3" s="9">
         <f t="shared" ref="BKL3:BKN3" si="634">BKK3</f>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BKM3" s="9">
         <f t="shared" si="634"/>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BKN3" s="9">
         <f t="shared" si="634"/>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BKO3" s="9">
         <f t="shared" ref="BKO3" si="635">BKN3</f>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BKP3" s="9">
         <f t="shared" ref="BKP3:BKS3" si="636">BKO3</f>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BKQ3" s="9">
         <f t="shared" si="636"/>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BKR3" s="9">
         <f t="shared" si="636"/>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BKS3" s="9">
         <f t="shared" si="636"/>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BKT3" s="9">
         <f t="shared" ref="BKT3" si="637">BKS3</f>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BKU3" s="9">
         <f t="shared" ref="BKU3" si="638">BKT3</f>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BKV3" s="9">
         <f t="shared" ref="BKV3" si="639">BKU3</f>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BKW3" s="9">
         <f t="shared" ref="BKW3" si="640">BKV3</f>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BKX3" s="9">
         <f t="shared" ref="BKX3:BLA3" si="641">BKW3</f>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BKY3" s="9">
         <f t="shared" si="641"/>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BKZ3" s="9">
         <f t="shared" si="641"/>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BLA3" s="9">
         <f t="shared" si="641"/>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BLB3" s="9">
         <f t="shared" ref="BLB3" si="642">BLA3</f>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BLC3" s="9">
         <f t="shared" ref="BLC3" si="643">BLB3</f>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BLD3" s="9">
         <f t="shared" ref="BLD3" si="644">BLC3</f>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BLE3" s="9">
         <f t="shared" ref="BLE3" si="645">BLD3</f>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BLF3" s="9">
         <f>BLE3</f>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BLG3" s="9">
         <f t="shared" ref="BLG3" si="646">BLF3</f>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BLH3" s="9">
         <f t="shared" ref="BLH3" si="647">BLG3</f>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BLI3" s="9">
         <f>BLH3</f>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BLJ3" s="9">
         <f t="shared" ref="BLJ3" si="648">BLI3</f>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BLK3" s="9">
         <f t="shared" ref="BLK3" si="649">BLJ3</f>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
       </c>
       <c r="BLL3" s="9">
         <f t="shared" ref="BLL3" si="650">BLK3</f>
-        <v>892.25409836065569</v>
+        <v>879.35526315789468</v>
+      </c>
+      <c r="BLM3" s="9">
+        <f t="shared" ref="BLM3" si="651">BLL3</f>
+        <v>879.35526315789468</v>
+      </c>
+      <c r="BLN3" s="9">
+        <f t="shared" ref="BLN3" si="652">BLM3</f>
+        <v>879.35526315789468</v>
+      </c>
+      <c r="BLO3" s="9">
+        <f t="shared" ref="BLO3" si="653">BLN3</f>
+        <v>879.35526315789468</v>
+      </c>
+      <c r="BLP3" s="9">
+        <f t="shared" ref="BLP3:BLS3" si="654">BLO3</f>
+        <v>879.35526315789468</v>
+      </c>
+      <c r="BLQ3" s="9">
+        <f t="shared" si="654"/>
+        <v>879.35526315789468</v>
+      </c>
+      <c r="BLR3" s="9">
+        <f t="shared" si="654"/>
+        <v>879.35526315789468</v>
+      </c>
+      <c r="BLS3" s="9">
+        <f t="shared" si="654"/>
+        <v>879.35526315789468</v>
       </c>
     </row>
-    <row r="4" spans="1:1676">
+    <row r="4" spans="1:1683">
       <c r="BEM4" s="15"/>
       <c r="BEN4" s="15"/>
       <c r="BEO4" s="15"/>

</xml_diff>